<commit_message>
add completed export files
</commit_message>
<xml_diff>
--- a/All_Monthly_Revenue.xlsx
+++ b/All_Monthly_Revenue.xlsx
@@ -2,28 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shary\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D9956A7A-DA43-46F9-93BD-BC0BADCF435F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C23BFB-0BC3-4BF1-B56A-E250F4938715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1576E16A-76CF-47AF-9CA7-19BFF1AE9FEC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1576E16A-76CF-47AF-9CA7-19BFF1AE9FEC}"/>
   </bookViews>
   <sheets>
-    <sheet name="All_Monthly_Revenue" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="All_Monthly_Revenue" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId2"/>
+    <pivotCache cacheId="67" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="8">
   <si>
     <t>State</t>
   </si>
@@ -48,17 +49,14 @@
   <si>
     <t>Grand Total</t>
   </si>
-  <si>
-    <t>Sum of Month</t>
-  </si>
-  <si>
-    <t>Sum of YEAR</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -492,7 +490,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -535,16 +533,21 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="42" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -572,6 +575,7 @@
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Currency" xfId="42" builtinId="4"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -601,23 +605,1096 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[All_Monthly_Revenue.xlsx]All_Monthly_Revenue!PivotTable19</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:ln w="28575" cap="rnd">
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="circle"/>
+          <c:size val="5"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>All_Monthly_Revenue!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>All_Monthly_Revenue!$F$3:$F$16</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="12"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>1</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>2</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>3</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>4</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>5</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>6</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>7</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>8</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>9</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>10</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>11</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>12</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>2025</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>All_Monthly_Revenue!$G$3:$G$16</c:f>
+              <c:numCache>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>150745.88</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>140234.23999999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>160846.60999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>156773.91</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>157710.74</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>170305.34</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>191697.95</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>174867.46</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>168503.25</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>277382.19</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>196108.93</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>186487.64</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-02BB-412D-8BB0-5BC055AB7B27}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1835646335"/>
+        <c:axId val="1835630975"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1835646335"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1835630975"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1835630975"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1835646335"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1409700</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3338411-9911-2F27-75D6-AB74601BCCB7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Sha'Rya Weaver" refreshedDate="46141.562669328705" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{D30FEB74-D1AA-4B8E-8EEF-0F29FB907FE4}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Sha'Rya Weaver" refreshedDate="46142.480577314818" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="12" xr:uid="{E405C171-C6C8-49C3-B305-948E5A60CC25}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:D49" sheet="All_Monthly_Revenue"/>
+    <worksheetSource ref="B1:D13" sheet="All_Monthly_Revenue"/>
   </cacheSource>
-  <cacheFields count="4">
-    <cacheField name="State" numFmtId="0">
-      <sharedItems count="1">
-        <s v="Massachusetts"/>
-      </sharedItems>
-    </cacheField>
+  <cacheFields count="3">
     <cacheField name="YEAR" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2022" maxValue="2025" count="4">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2025" maxValue="2025" count="1">
         <n v="2025"/>
-        <n v="2024"/>
-        <n v="2023"/>
-        <n v="2022"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Month" numFmtId="0">
@@ -636,55 +1713,8 @@
         <n v="1"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="MonthlyRevenue" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="58716.74" maxValue="277382.19" count="46">
-        <n v="186487.64"/>
-        <n v="196108.93"/>
-        <n v="277382.19"/>
-        <n v="168503.25"/>
-        <n v="174867.46"/>
-        <n v="191697.95"/>
-        <n v="170305.34"/>
-        <n v="157710.74"/>
-        <n v="156773.91"/>
-        <n v="160846.60999999999"/>
-        <n v="140234.23999999999"/>
-        <n v="150745.88"/>
-        <n v="139388.56"/>
-        <n v="96729.12"/>
-        <n v="110582.18"/>
-        <n v="111867.1"/>
-        <n v="123926.2"/>
-        <n v="126212.14"/>
-        <n v="116310.73"/>
-        <n v="106193.39"/>
-        <n v="107421.88"/>
-        <n v="110968.54"/>
-        <n v="103968.7"/>
-        <n v="117915.05"/>
-        <n v="101641.22"/>
-        <n v="105670.08"/>
-        <n v="113824.37"/>
-        <n v="121968.93"/>
-        <n v="120793.96"/>
-        <n v="101710.16"/>
-        <n v="109021.42"/>
-        <n v="109369"/>
-        <n v="112443.92"/>
-        <n v="104454.67"/>
-        <n v="70025.64"/>
-        <n v="70654.73"/>
-        <n v="72514.81"/>
-        <n v="58716.74"/>
-        <n v="73543.48"/>
-        <n v="67271.23"/>
-        <n v="81227.820000000007"/>
-        <n v="75919.64"/>
-        <n v="81333.600000000006"/>
-        <n v="77390"/>
-        <n v="65616"/>
-        <n v="69396.42"/>
-      </sharedItems>
+    <cacheField name="MonthlyRevenue" numFmtId="44">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="140234.23999999999" maxValue="277382.19"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -696,416 +1726,164 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="48">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="12">
   <r>
     <x v="0"/>
     <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="2"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="3"/>
-    <x v="3"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="4"/>
-    <x v="4"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="5"/>
-    <x v="5"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="6"/>
-    <x v="6"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="7"/>
-    <x v="7"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="8"/>
-    <x v="8"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="9"/>
-    <x v="9"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="10"/>
-    <x v="10"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="11"/>
-    <x v="11"/>
+    <n v="186487.64"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <x v="0"/>
-    <x v="12"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="13"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="2"/>
-    <x v="14"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="3"/>
-    <x v="15"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="4"/>
-    <x v="16"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="5"/>
-    <x v="17"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="6"/>
-    <x v="18"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="7"/>
-    <x v="19"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="8"/>
-    <x v="20"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="9"/>
-    <x v="21"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="10"/>
-    <x v="22"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="1"/>
-    <x v="11"/>
-    <x v="23"/>
+    <n v="196108.93"/>
   </r>
   <r>
     <x v="0"/>
     <x v="2"/>
-    <x v="0"/>
-    <x v="24"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="1"/>
-    <x v="25"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="26"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="3"/>
-    <x v="27"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="4"/>
-    <x v="17"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="5"/>
-    <x v="28"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="6"/>
-    <x v="29"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="7"/>
-    <x v="30"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="8"/>
-    <x v="31"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="9"/>
-    <x v="32"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="10"/>
-    <x v="33"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <x v="11"/>
-    <x v="12"/>
+    <n v="277382.19"/>
   </r>
   <r>
     <x v="0"/>
     <x v="3"/>
-    <x v="0"/>
-    <x v="34"/>
+    <n v="168503.25"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="1"/>
-    <x v="35"/>
+    <x v="4"/>
+    <n v="174867.46"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="2"/>
-    <x v="36"/>
+    <x v="5"/>
+    <n v="191697.95"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="37"/>
+    <x v="6"/>
+    <n v="170305.34"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="4"/>
-    <x v="38"/>
+    <x v="7"/>
+    <n v="157710.74"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="5"/>
-    <x v="39"/>
+    <x v="8"/>
+    <n v="156773.91"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="6"/>
-    <x v="40"/>
+    <x v="9"/>
+    <n v="160846.60999999999"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="7"/>
-    <x v="41"/>
+    <x v="10"/>
+    <n v="140234.23999999999"/>
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
-    <x v="8"/>
-    <x v="42"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="3"/>
-    <x v="9"/>
-    <x v="43"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="3"/>
-    <x v="10"/>
-    <x v="44"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="3"/>
     <x v="11"/>
-    <x v="45"/>
+    <n v="150745.88"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EBC28679-AAAD-4D73-AAC5-FB55008733CC}" name="PivotTable2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="H4:K6" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A282739A-724B-4482-A830-21880A96EB00}" name="PivotTable19" cacheId="67" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+  <location ref="F2:G16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
       <items count="2">
         <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField dataField="1" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="5">
-        <item h="1" x="3"/>
-        <item h="1" x="2"/>
-        <item h="1" x="1"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="13">
+        <item x="11"/>
+        <item x="10"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
         <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField dataField="1" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="13">
-        <item h="1" x="11"/>
-        <item h="1" x="10"/>
-        <item h="1" x="9"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="6"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="3"/>
-        <item h="1" x="2"/>
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0">
-      <items count="47">
-        <item x="37"/>
-        <item x="44"/>
-        <item x="39"/>
-        <item x="45"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="38"/>
-        <item x="41"/>
-        <item x="43"/>
-        <item x="40"/>
-        <item x="42"/>
-        <item x="13"/>
-        <item x="24"/>
-        <item x="29"/>
-        <item x="22"/>
-        <item x="33"/>
-        <item x="25"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="14"/>
-        <item x="21"/>
-        <item x="15"/>
-        <item x="32"/>
-        <item x="26"/>
-        <item x="18"/>
-        <item x="23"/>
-        <item x="28"/>
-        <item x="27"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="12"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="8"/>
-        <item x="7"/>
-        <item x="9"/>
-        <item x="3"/>
-        <item x="6"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField dataField="1" numFmtId="44" showAll="0"/>
   </pivotFields>
-  <rowFields count="1">
+  <rowFields count="2">
     <field x="0"/>
+    <field x="1"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="14">
     <i>
       <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
     </i>
     <i t="grand">
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
+  <colItems count="1">
+    <i/>
   </colItems>
-  <dataFields count="3">
-    <dataField name="Sum of YEAR" fld="1" baseField="0" baseItem="0"/>
-    <dataField name="Sum of Month" fld="2" baseField="0" baseItem="0"/>
-    <dataField name="Sum of MonthlyRevenue" fld="3" baseField="0" baseItem="0"/>
+  <dataFields count="1">
+    <dataField name="Sum of MonthlyRevenue" fld="2" baseField="0" baseItem="0" numFmtId="44"/>
   </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -1116,6 +1894,26 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69927C9C-9727-4EC3-8AE1-ED03747B7383}" name="Table1" displayName="Table1" ref="A1:D49" totalsRowShown="0">
+  <autoFilter ref="A1:D49" xr:uid="{69927C9C-9727-4EC3-8AE1-ED03747B7383}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="2024"/>
+        <filter val="2025"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{ACAA39DA-0378-4704-B33D-6C1AD0F13061}" name="State"/>
+    <tableColumn id="2" xr3:uid="{6BD9538E-EF5A-4190-9F4C-F6F2B9508D38}" name="YEAR"/>
+    <tableColumn id="3" xr3:uid="{1AD31343-3277-4F65-8844-FCAEFABB1A86}" name="Month"/>
+    <tableColumn id="4" xr3:uid="{19CE8594-A1B6-45C1-9164-335FA92C7FB6}" name="MonthlyRevenue"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1434,33 +2232,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA63C00-F022-4637-9DE8-775EEF40AD6B}">
-  <dimension ref="A1:K49"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E995C9E-55DF-41C4-B734-F4F9D03646FC}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="20" width="10" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11" bestFit="1" customWidth="1"/>
-    <col min="22" max="24" width="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7" bestFit="1" customWidth="1"/>
-    <col min="26" max="33" width="10" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="9" bestFit="1" customWidth="1"/>
-    <col min="37" max="41" width="10" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="9" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="9" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="11" bestFit="1" customWidth="1"/>
-    <col min="48" max="59" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDA63C00-F022-4637-9DE8-775EEF40AD6B}">
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" customWidth="1"/>
+    <col min="10" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="15" width="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="10" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="29" width="10" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="10" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9" bestFit="1" customWidth="1"/>
+    <col min="34" max="39" width="10" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9" bestFit="1" customWidth="1"/>
+    <col min="41" max="54" width="10" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="56" max="59" width="10" bestFit="1" customWidth="1"/>
     <col min="60" max="61" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1474,7 +2289,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1484,11 +2299,17 @@
       <c r="C2">
         <v>12</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="4">
         <v>186487.64</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1498,11 +2319,17 @@
       <c r="C3">
         <v>11</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="4">
         <v>196108.93</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F3" s="2">
+        <v>2025</v>
+      </c>
+      <c r="G3" s="5">
+        <v>2131664.1399999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1512,23 +2339,17 @@
       <c r="C4">
         <v>10</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="4">
         <v>277382.19</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" t="s">
-        <v>9</v>
-      </c>
-      <c r="J4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5">
+        <v>150745.88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1538,23 +2359,17 @@
       <c r="C5">
         <v>9</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="4">
         <v>168503.25</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I5" s="3">
-        <v>97128</v>
-      </c>
-      <c r="J5" s="3">
-        <v>312</v>
-      </c>
-      <c r="K5" s="3">
-        <v>5733256.2700000014</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F5" s="3">
+        <v>2</v>
+      </c>
+      <c r="G5" s="5">
+        <v>140234.23999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1564,23 +2379,17 @@
       <c r="C6">
         <v>8</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="4">
         <v>174867.46</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="3">
-        <v>97128</v>
-      </c>
-      <c r="J6" s="3">
-        <v>312</v>
-      </c>
-      <c r="K6" s="3">
-        <v>5733256.2700000014</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F6" s="3">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5">
+        <v>160846.60999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1590,11 +2399,17 @@
       <c r="C7">
         <v>7</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="4">
         <v>191697.95</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F7" s="3">
+        <v>4</v>
+      </c>
+      <c r="G7" s="5">
+        <v>156773.91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1604,11 +2419,17 @@
       <c r="C8">
         <v>6</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="4">
         <v>170305.34</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F8" s="3">
+        <v>5</v>
+      </c>
+      <c r="G8" s="5">
+        <v>157710.74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1618,11 +2439,17 @@
       <c r="C9">
         <v>5</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="4">
         <v>157710.74</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F9" s="3">
+        <v>6</v>
+      </c>
+      <c r="G9" s="5">
+        <v>170305.34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1632,11 +2459,17 @@
       <c r="C10">
         <v>4</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="4">
         <v>156773.91</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F10" s="3">
+        <v>7</v>
+      </c>
+      <c r="G10" s="5">
+        <v>191697.95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1646,11 +2479,17 @@
       <c r="C11">
         <v>3</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="4">
         <v>160846.60999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F11" s="3">
+        <v>8</v>
+      </c>
+      <c r="G11" s="5">
+        <v>174867.46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1660,11 +2499,17 @@
       <c r="C12">
         <v>2</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="4">
         <v>140234.23999999999</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F12" s="3">
+        <v>9</v>
+      </c>
+      <c r="G12" s="5">
+        <v>168503.25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1674,11 +2519,17 @@
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="4">
         <v>150745.88</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F13" s="3">
+        <v>10</v>
+      </c>
+      <c r="G13" s="5">
+        <v>277382.19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1688,11 +2539,17 @@
       <c r="C14">
         <v>12</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="4">
         <v>139388.56</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F14" s="3">
+        <v>11</v>
+      </c>
+      <c r="G14" s="5">
+        <v>196108.93</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1702,11 +2559,17 @@
       <c r="C15">
         <v>11</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="4">
         <v>96729.12</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F15" s="3">
+        <v>12</v>
+      </c>
+      <c r="G15" s="5">
+        <v>186487.64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1716,8 +2579,14 @@
       <c r="C16">
         <v>10</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="4">
         <v>110582.18</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="5">
+        <v>2131664.1399999997</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1730,7 +2599,7 @@
       <c r="C17">
         <v>9</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="4">
         <v>111867.1</v>
       </c>
     </row>
@@ -1744,7 +2613,7 @@
       <c r="C18">
         <v>8</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="4">
         <v>123926.2</v>
       </c>
     </row>
@@ -1758,7 +2627,7 @@
       <c r="C19">
         <v>7</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="4">
         <v>126212.14</v>
       </c>
     </row>
@@ -1772,7 +2641,7 @@
       <c r="C20">
         <v>6</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="4">
         <v>116310.73</v>
       </c>
     </row>
@@ -1786,7 +2655,7 @@
       <c r="C21">
         <v>5</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="4">
         <v>106193.39</v>
       </c>
     </row>
@@ -1800,7 +2669,7 @@
       <c r="C22">
         <v>4</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="4">
         <v>107421.88</v>
       </c>
     </row>
@@ -1814,7 +2683,7 @@
       <c r="C23">
         <v>3</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="4">
         <v>110968.54</v>
       </c>
     </row>
@@ -1828,7 +2697,7 @@
       <c r="C24">
         <v>2</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="4">
         <v>103968.7</v>
       </c>
     </row>
@@ -1842,11 +2711,11 @@
       <c r="C25">
         <v>1</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="4">
         <v>117915.05</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1860,7 +2729,7 @@
         <v>101641.22</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1874,7 +2743,7 @@
         <v>105670.08</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1888,7 +2757,7 @@
         <v>113824.37</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1902,7 +2771,7 @@
         <v>121968.93</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1916,7 +2785,7 @@
         <v>126212.14</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1930,7 +2799,7 @@
         <v>120793.96</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -1944,7 +2813,7 @@
         <v>101710.16</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -1958,7 +2827,7 @@
         <v>109021.42</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -1972,7 +2841,7 @@
         <v>109369</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -1986,7 +2855,7 @@
         <v>112443.92</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>4</v>
       </c>
@@ -2000,7 +2869,7 @@
         <v>104454.67</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -2014,7 +2883,7 @@
         <v>139388.56</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -2028,7 +2897,7 @@
         <v>70025.64</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -2042,7 +2911,7 @@
         <v>70654.73</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -2056,7 +2925,7 @@
         <v>72514.81</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -2070,7 +2939,7 @@
         <v>58716.74</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -2084,7 +2953,7 @@
         <v>73543.48</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -2098,7 +2967,7 @@
         <v>67271.23</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -2112,7 +2981,7 @@
         <v>81227.820000000007</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -2126,7 +2995,7 @@
         <v>75919.64</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -2140,7 +3009,7 @@
         <v>81333.600000000006</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -2154,7 +3023,7 @@
         <v>77390</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -2168,7 +3037,7 @@
         <v>65616</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -2184,5 +3053,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>